<commit_message>
Initial commit from workspace
</commit_message>
<xml_diff>
--- a/output/screening_results.xlsx
+++ b/output/screening_results.xlsx
@@ -424,7 +424,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Resume</t>
+          <t>Candidate</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -444,7 +444,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Rohan_Mehta_Resume.pdf</t>
+          <t>Rohan Mehta</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -462,7 +462,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Rahul_Sharma_Resume.pdf</t>
+          <t>Rahul Sharma</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -480,7 +480,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Anil_Kumar_Resume.pdf</t>
+          <t>Anil Kumar</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -498,7 +498,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Akash_Jain_Resume.pdf</t>
+          <t>Akash Jain</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -516,7 +516,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Sanjay_Reddy_Resume.pdf</t>
+          <t>Sanjay Reddy</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -534,7 +534,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Monika_Agarwal_Resume.pdf</t>
+          <t>Monika Agarwal</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -552,7 +552,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Aditya_Menon_Resume.pdf</t>
+          <t>Aditya Menon</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -570,7 +570,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Kiran_Malhotra_Resume.pdf</t>
+          <t>Kiran Malhotra</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -588,7 +588,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Nisha_Gupta_Resume.pdf</t>
+          <t>Nisha Gupta</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -606,7 +606,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Farhan_Ali_Resume.pdf</t>
+          <t>Farhan Ali</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -624,7 +624,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Deepika_Nair_Resume.pdf</t>
+          <t>Deepika Nair</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -642,7 +642,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Gaurav_Mishra_Resume.pdf</t>
+          <t>Gaurav Mishra</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -660,7 +660,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Harish_Babu_Resume.pdf</t>
+          <t>Harish Babu</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -678,7 +678,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Lokesh_Kumar_Resume.pdf</t>
+          <t>Lokesh Kumar</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -696,7 +696,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Priya_Nair_Resume.pdf</t>
+          <t>Priya Nair</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -714,7 +714,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Bhavana_Rao_Resume.pdf</t>
+          <t>Bhavana Rao</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -732,7 +732,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Chirag_Shah_Resume.pdf</t>
+          <t>Chirag Shah</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -750,7 +750,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Sneha_Rao_Resume.pdf</t>
+          <t>Sneha Rao</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -768,7 +768,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Divya_Krishnan_Resume.pdf</t>
+          <t>Divya Krishnan</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -786,7 +786,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Neha_Singh_Resume.pdf</t>
+          <t>Neha Singh</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -804,7 +804,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Arjun_Verma_Resume.pdf</t>
+          <t>Arjun Verma</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -822,7 +822,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ritika_Sinha_Resume.pdf</t>
+          <t>Ritika Sinha</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -840,7 +840,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Yash_Patel_Resume.pdf</t>
+          <t>Yash Patel</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Vikram_Patel_Resume.pdf</t>
+          <t>Vikram Patel</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -876,7 +876,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Kavya_Iyer_Resume.pdf</t>
+          <t>Kavya Iyer</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -894,7 +894,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Manoj_Kulkarni_Resume.pdf</t>
+          <t>Manoj Kulkarni</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -912,7 +912,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Meera_Joshi_Resume.pdf</t>
+          <t>Meera Joshi</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -930,7 +930,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Pooja_Desai_Resume.pdf</t>
+          <t>Pooja Desai</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -948,7 +948,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Aisha_Khan_Resume.pdf</t>
+          <t>Aisha Khan</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -966,7 +966,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Ishita_Roy_Resume.pdf</t>
+          <t>Ishita Roy</t>
         </is>
       </c>
       <c r="C31" t="n">

</xml_diff>